<commit_message>
Implementa correcao nas contas dos IPS
</commit_message>
<xml_diff>
--- a/ProjetoRedes.xlsx
+++ b/ProjetoRedes.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Desktop\ProjetoRedes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\Desktop\ProjetoRedes\Projeto-de-Redes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{289302B0-FFBF-49F6-95F5-E1E31D706EC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21BA7E75-E74B-4B6A-A8DE-B80C470ED696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="166">
   <si>
     <t>AVEIRO</t>
   </si>
@@ -140,9 +140,6 @@
     <t>10.99.9.97</t>
   </si>
   <si>
-    <t>10.99.9.126</t>
-  </si>
-  <si>
     <t>10.99.9.127</t>
   </si>
   <si>
@@ -203,9 +200,6 @@
     <t>COVILHA</t>
   </si>
   <si>
-    <t>10.30.0.0</t>
-  </si>
-  <si>
     <t>10.30.0.1</t>
   </si>
   <si>
@@ -215,18 +209,12 @@
     <t>10.30.0.63</t>
   </si>
   <si>
-    <t>10.30.0.64</t>
-  </si>
-  <si>
     <t>10.30.0.126</t>
   </si>
   <si>
     <t>10.30.0.127</t>
   </si>
   <si>
-    <t>10.30.0.128</t>
-  </si>
-  <si>
     <t>10.30.0.190</t>
   </si>
   <si>
@@ -236,9 +224,6 @@
     <t>10.30.0.191</t>
   </si>
   <si>
-    <t>10.30.0.192</t>
-  </si>
-  <si>
     <t>10.30.0.222</t>
   </si>
   <si>
@@ -248,16 +233,10 @@
     <t>10.30.0.223</t>
   </si>
   <si>
-    <t>10.30.0.224</t>
-  </si>
-  <si>
     <t>10.30.0.238</t>
   </si>
   <si>
     <t>10.30.0.239</t>
-  </si>
-  <si>
-    <t>10.30.0.240</t>
   </si>
   <si>
     <t>COVILLHA</t>
@@ -609,6 +588,24 @@
   </si>
   <si>
     <t>10.30.0.255</t>
+  </si>
+  <si>
+    <t>10.30.9.0</t>
+  </si>
+  <si>
+    <t>10.30.9.64</t>
+  </si>
+  <si>
+    <t>10.30.9.128</t>
+  </si>
+  <si>
+    <t>10.30.9.192</t>
+  </si>
+  <si>
+    <t>10.30.9.224</t>
+  </si>
+  <si>
+    <t>10.30.9.240</t>
   </si>
 </sst>
 </file>
@@ -694,7 +691,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -749,12 +746,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -783,7 +774,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -853,9 +844,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1419,11 +1407,12 @@
       <c r="K5" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="L5" s="10" t="s">
+      <c r="L5" s="10" t="str">
+        <f>+H15</f>
+        <v>MANAGMENT</v>
+      </c>
+      <c r="M5" s="12" t="s">
         <v>34</v>
-      </c>
-      <c r="M5" s="12" t="s">
-        <v>35</v>
       </c>
       <c r="N5" s="2"/>
       <c r="O5" s="6" t="s">
@@ -1449,7 +1438,7 @@
     </row>
     <row r="6" spans="1:21" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B6" s="10">
         <v>15</v>
@@ -1468,26 +1457,26 @@
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="I6" s="10" t="s">
         <v>36</v>
-      </c>
-      <c r="I6" s="10" t="s">
-        <v>37</v>
       </c>
       <c r="J6" s="10" t="s">
         <v>27</v>
       </c>
       <c r="K6" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="L6" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="L6" s="10" t="s">
+      <c r="M6" s="12" t="s">
         <v>39</v>
-      </c>
-      <c r="M6" s="12" t="s">
-        <v>40</v>
       </c>
       <c r="N6" s="2"/>
       <c r="O6" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P6" s="6">
         <v>128</v>
@@ -1509,7 +1498,7 @@
     </row>
     <row r="7" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B7" s="10">
         <v>7</v>
@@ -1518,36 +1507,36 @@
         <v>9</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E7" s="10">
         <v>14</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G7" s="1"/>
       <c r="H7" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I7" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="J7" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="J7" s="10" t="s">
+      <c r="K7" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="K7" s="10" t="s">
+      <c r="L7" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="L7" s="10" t="s">
+      <c r="M7" s="10" t="s">
         <v>47</v>
-      </c>
-      <c r="M7" s="10" t="s">
-        <v>48</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="P7" s="6">
         <v>160</v>
@@ -1569,7 +1558,7 @@
     </row>
     <row r="8" spans="1:21" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B8" s="10">
         <v>7</v>
@@ -1578,36 +1567,36 @@
         <v>9</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E8" s="10">
         <v>14</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G8" s="1"/>
       <c r="H8" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="I8" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="J8" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="K8" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="J8" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="K8" s="10" t="s">
+      <c r="L8" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="L8" s="10" t="s">
+      <c r="M8" s="10" t="s">
         <v>52</v>
-      </c>
-      <c r="M8" s="10" t="s">
-        <v>53</v>
       </c>
       <c r="N8" s="2"/>
       <c r="O8" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="P8" s="6">
         <v>176</v>
@@ -1629,7 +1618,7 @@
     <row r="9" spans="1:21" ht="0.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="G9" s="1"/>
       <c r="O9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="Q9">
         <f>256-14</f>
@@ -1675,7 +1664,7 @@
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
       <c r="G12" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="3"/>
@@ -1772,19 +1761,19 @@
         <v>23</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>55</v>
+        <v>160</v>
       </c>
       <c r="J14" s="10" t="s">
         <v>19</v>
       </c>
       <c r="K14" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="L14" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="M14" s="10" t="s">
         <v>56</v>
-      </c>
-      <c r="L14" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="M14" s="10" t="s">
-        <v>58</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="11" t="s">
@@ -1810,7 +1799,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B15" s="10">
         <v>33</v>
@@ -1830,26 +1819,26 @@
       </c>
       <c r="G15" s="2"/>
       <c r="H15" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>59</v>
+        <v>161</v>
       </c>
       <c r="J15" s="10" t="s">
         <v>19</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="P15" s="6">
         <v>64</v>
@@ -1871,7 +1860,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B16" s="10">
         <v>31</v>
@@ -1891,26 +1880,26 @@
       </c>
       <c r="G16" s="2"/>
       <c r="H16" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>62</v>
+        <v>162</v>
       </c>
       <c r="J16" s="10" t="s">
         <v>19</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="L16" s="10" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="M16" s="10" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P16" s="6">
         <v>128</v>
@@ -1932,7 +1921,7 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A17" s="9" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B17" s="10">
         <v>15</v>
@@ -1952,26 +1941,26 @@
       </c>
       <c r="G17" s="2"/>
       <c r="H17" s="9" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>66</v>
+        <v>163</v>
       </c>
       <c r="J17" s="10" t="s">
         <v>27</v>
       </c>
       <c r="K17" s="10" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="L17" s="10" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="M17" s="12" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="11" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="P17" s="6">
         <v>192</v>
@@ -1993,7 +1982,7 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B18" s="10">
         <v>12</v>
@@ -2002,7 +1991,7 @@
         <v>14</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E18" s="10">
         <v>14</v>
@@ -2013,26 +2002,26 @@
       </c>
       <c r="G18" s="2"/>
       <c r="H18" s="9" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>70</v>
+        <v>164</v>
       </c>
       <c r="J18" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="K18" s="10" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="L18" s="10" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="M18" s="10" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="11" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="P18" s="6">
         <v>224</v>
@@ -2054,7 +2043,7 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B19" s="10">
         <v>9</v>
@@ -2063,7 +2052,7 @@
         <v>11</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E19" s="10">
         <v>14</v>
@@ -2074,26 +2063,26 @@
       </c>
       <c r="G19" s="2"/>
       <c r="H19" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>73</v>
+        <v>165</v>
       </c>
       <c r="J19" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="K19" s="10" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="L19" s="10" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="M19" s="10" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="P19" s="6">
         <v>240</v>
@@ -2149,7 +2138,7 @@
       <c r="H21" s="13"/>
       <c r="I21" s="13"/>
       <c r="J21" s="19" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="K21" s="13"/>
       <c r="L21" s="13"/>
@@ -2165,36 +2154,36 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A22" s="14" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="E22" s="14" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="F22" s="13"/>
       <c r="G22" s="13"/>
       <c r="H22" s="14" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="I22" s="14" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="J22" s="14" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="K22" s="14" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="L22" s="14" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="M22" s="13"/>
       <c r="N22" s="13"/>
@@ -2208,36 +2197,36 @@
     </row>
     <row r="23" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="15" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="F23" s="13"/>
       <c r="G23" s="13"/>
       <c r="H23" s="15" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="I23" s="16" t="s">
-        <v>81</v>
-      </c>
-      <c r="J23" s="25" t="s">
-        <v>86</v>
+        <v>74</v>
+      </c>
+      <c r="J23" s="15" t="s">
+        <v>79</v>
       </c>
       <c r="K23" s="15" t="s">
-        <v>83</v>
-      </c>
-      <c r="L23" s="25" t="s">
-        <v>84</v>
+        <v>76</v>
+      </c>
+      <c r="L23" s="15" t="s">
+        <v>77</v>
       </c>
       <c r="M23" s="13"/>
       <c r="N23" s="13"/>
@@ -2251,34 +2240,34 @@
     </row>
     <row r="24" spans="1:21" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="B24" s="15" t="s">
         <v>80</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>87</v>
       </c>
       <c r="C24" s="15"/>
       <c r="D24" s="15" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="F24" s="13"/>
       <c r="G24" s="13"/>
       <c r="H24" s="17" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="I24" s="15" t="s">
-        <v>89</v>
-      </c>
-      <c r="J24" s="25" t="s">
-        <v>90</v>
+        <v>82</v>
+      </c>
+      <c r="J24" s="15" t="s">
+        <v>83</v>
       </c>
       <c r="K24" s="15" t="s">
-        <v>83</v>
-      </c>
-      <c r="L24" s="25" t="s">
-        <v>84</v>
+        <v>76</v>
+      </c>
+      <c r="L24" s="15" t="s">
+        <v>77</v>
       </c>
       <c r="M24" s="13"/>
       <c r="N24" s="13"/>
@@ -2292,34 +2281,34 @@
     </row>
     <row r="25" spans="1:21" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="17" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="C25" s="15"/>
       <c r="D25" s="15" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="F25" s="13"/>
       <c r="G25" s="13"/>
       <c r="H25" s="17" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="I25" s="15" t="s">
-        <v>92</v>
-      </c>
-      <c r="J25" s="25" t="s">
-        <v>93</v>
+        <v>85</v>
+      </c>
+      <c r="J25" s="15" t="s">
+        <v>86</v>
       </c>
       <c r="K25" s="15" t="s">
-        <v>94</v>
-      </c>
-      <c r="L25" s="25" t="s">
-        <v>84</v>
+        <v>87</v>
+      </c>
+      <c r="L25" s="15" t="s">
+        <v>77</v>
       </c>
       <c r="M25" s="13"/>
       <c r="N25" s="13"/>
@@ -2333,36 +2322,36 @@
     </row>
     <row r="26" spans="1:21" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="15" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="F26" s="13"/>
       <c r="G26" s="13"/>
       <c r="H26" s="17" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="I26" s="15" t="s">
-        <v>97</v>
-      </c>
-      <c r="J26" s="25" t="s">
-        <v>98</v>
+        <v>90</v>
+      </c>
+      <c r="J26" s="15" t="s">
+        <v>91</v>
       </c>
       <c r="K26" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="L26" s="25" t="s">
-        <v>84</v>
+        <v>44</v>
+      </c>
+      <c r="L26" s="15" t="s">
+        <v>77</v>
       </c>
       <c r="M26" s="13"/>
       <c r="N26" s="13"/>
@@ -2376,36 +2365,36 @@
     </row>
     <row r="27" spans="1:21" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="15" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E27" s="15" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="F27" s="13"/>
       <c r="G27" s="13"/>
       <c r="H27" s="17" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="I27" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="J27" s="25" t="s">
-        <v>100</v>
+        <v>92</v>
+      </c>
+      <c r="J27" s="15" t="s">
+        <v>93</v>
       </c>
       <c r="K27" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="L27" s="25" t="s">
-        <v>84</v>
+      <c r="L27" s="15" t="s">
+        <v>77</v>
       </c>
       <c r="M27" s="13"/>
       <c r="N27" s="13"/>
@@ -2419,10 +2408,10 @@
     </row>
     <row r="28" spans="1:21" ht="24.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="15" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="C28" s="15" t="s">
         <v>28</v>
@@ -2431,24 +2420,24 @@
         <v>27</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="F28" s="13"/>
       <c r="G28" s="13"/>
       <c r="H28" s="17" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="I28" s="15" t="s">
-        <v>101</v>
-      </c>
-      <c r="J28" s="25" t="s">
-        <v>102</v>
+        <v>94</v>
+      </c>
+      <c r="J28" s="15" t="s">
+        <v>95</v>
       </c>
       <c r="K28" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="L28" s="25" t="s">
-        <v>84</v>
+      <c r="L28" s="15" t="s">
+        <v>77</v>
       </c>
       <c r="M28" s="13"/>
       <c r="N28" s="13"/>
@@ -2462,10 +2451,10 @@
     </row>
     <row r="29" spans="1:21" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="15" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="C29" s="15" t="s">
         <v>20</v>
@@ -2474,24 +2463,24 @@
         <v>19</v>
       </c>
       <c r="E29" s="15" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="F29" s="13"/>
       <c r="G29" s="13"/>
       <c r="H29" s="17" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="I29" s="15" t="s">
-        <v>104</v>
-      </c>
-      <c r="J29" s="25" t="s">
-        <v>105</v>
+        <v>97</v>
+      </c>
+      <c r="J29" s="15" t="s">
+        <v>98</v>
       </c>
       <c r="K29" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="L29" s="25" t="s">
-        <v>84</v>
+      <c r="L29" s="15" t="s">
+        <v>77</v>
       </c>
       <c r="M29" s="13"/>
       <c r="N29" s="13"/>
@@ -2505,36 +2494,36 @@
     </row>
     <row r="30" spans="1:21" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="15" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D30" s="15" t="s">
         <v>27</v>
       </c>
       <c r="E30" s="15" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="F30" s="13"/>
       <c r="G30" s="13"/>
       <c r="H30" s="17" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="I30" s="15" t="s">
-        <v>106</v>
-      </c>
-      <c r="J30" s="25" t="s">
-        <v>107</v>
+        <v>99</v>
+      </c>
+      <c r="J30" s="15" t="s">
+        <v>100</v>
       </c>
       <c r="K30" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="L30" s="25" t="s">
-        <v>84</v>
+      <c r="L30" s="15" t="s">
+        <v>77</v>
       </c>
       <c r="M30" s="13"/>
       <c r="N30" s="13"/>
@@ -2548,36 +2537,36 @@
     </row>
     <row r="31" spans="1:21" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="15" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E31" s="15" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="F31" s="13"/>
       <c r="G31" s="13"/>
       <c r="H31" s="17" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="I31" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="J31" s="25" t="s">
-        <v>110</v>
+        <v>102</v>
+      </c>
+      <c r="J31" s="15" t="s">
+        <v>103</v>
       </c>
       <c r="K31" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="L31" s="25" t="s">
-        <v>84</v>
+        <v>44</v>
+      </c>
+      <c r="L31" s="15" t="s">
+        <v>77</v>
       </c>
       <c r="M31" s="13"/>
       <c r="N31" s="13"/>
@@ -2591,10 +2580,10 @@
     </row>
     <row r="32" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="15" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="C32" s="15" t="s">
         <v>33</v>
@@ -2603,24 +2592,24 @@
         <v>27</v>
       </c>
       <c r="E32" s="15" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="F32" s="13"/>
       <c r="G32" s="13"/>
       <c r="H32" s="17" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="I32" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="J32" s="25" t="s">
-        <v>114</v>
+        <v>106</v>
+      </c>
+      <c r="J32" s="15" t="s">
+        <v>107</v>
       </c>
       <c r="K32" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="L32" s="25" t="s">
-        <v>105</v>
+      <c r="L32" s="15" t="s">
+        <v>98</v>
       </c>
       <c r="M32" s="13"/>
       <c r="N32" s="13"/>
@@ -2634,36 +2623,36 @@
     </row>
     <row r="33" spans="1:21" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="15" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="E33" s="15" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="F33" s="13"/>
       <c r="G33" s="13"/>
       <c r="H33" s="17" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="I33" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="J33" s="25" t="s">
-        <v>117</v>
+        <v>106</v>
+      </c>
+      <c r="J33" s="15" t="s">
+        <v>110</v>
       </c>
       <c r="K33" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="L33" s="25" t="s">
-        <v>105</v>
+      <c r="L33" s="15" t="s">
+        <v>98</v>
       </c>
       <c r="M33" s="13"/>
       <c r="N33" s="13"/>
@@ -2677,36 +2666,36 @@
     </row>
     <row r="34" spans="1:21" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="15" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="D34" s="15" t="s">
         <v>27</v>
       </c>
       <c r="E34" s="15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F34" s="13"/>
       <c r="G34" s="13"/>
       <c r="H34" s="17" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="I34" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="J34" s="25" t="s">
-        <v>121</v>
+        <v>106</v>
+      </c>
+      <c r="J34" s="15" t="s">
+        <v>114</v>
       </c>
       <c r="K34" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="L34" s="25" t="s">
-        <v>105</v>
+      <c r="L34" s="15" t="s">
+        <v>98</v>
       </c>
       <c r="M34" s="13"/>
       <c r="N34" s="13"/>
@@ -2720,36 +2709,36 @@
     </row>
     <row r="35" spans="1:21" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="17" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="D35" s="15" t="s">
         <v>27</v>
       </c>
       <c r="E35" s="15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F35" s="13"/>
       <c r="G35" s="13"/>
       <c r="H35" s="17" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="I35" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="J35" s="25" t="s">
-        <v>125</v>
+        <v>106</v>
+      </c>
+      <c r="J35" s="15" t="s">
+        <v>118</v>
       </c>
       <c r="K35" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="L35" s="25" t="s">
-        <v>105</v>
+      <c r="L35" s="15" t="s">
+        <v>98</v>
       </c>
       <c r="M35" s="13"/>
       <c r="N35" s="13"/>
@@ -2763,36 +2752,36 @@
     </row>
     <row r="36" spans="1:21" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="17" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="D36" s="15" t="s">
         <v>27</v>
       </c>
       <c r="E36" s="15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F36" s="13"/>
       <c r="G36" s="13"/>
       <c r="H36" s="17" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="I36" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="J36" s="25" t="s">
-        <v>129</v>
+        <v>106</v>
+      </c>
+      <c r="J36" s="15" t="s">
+        <v>122</v>
       </c>
       <c r="K36" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="L36" s="25" t="s">
-        <v>105</v>
+      <c r="L36" s="15" t="s">
+        <v>98</v>
       </c>
       <c r="M36" s="13"/>
       <c r="N36" s="13"/>
@@ -2806,36 +2795,36 @@
     </row>
     <row r="37" spans="1:21" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="17" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D37" s="15" t="s">
         <v>27</v>
       </c>
       <c r="E37" s="15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F37" s="13"/>
       <c r="G37" s="13"/>
       <c r="H37" s="17" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="I37" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="J37" s="25" t="s">
-        <v>133</v>
+        <v>106</v>
+      </c>
+      <c r="J37" s="15" t="s">
+        <v>126</v>
       </c>
       <c r="K37" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="L37" s="25" t="s">
-        <v>105</v>
+      <c r="L37" s="15" t="s">
+        <v>98</v>
       </c>
       <c r="M37" s="13"/>
       <c r="N37" s="13"/>
@@ -2849,36 +2838,36 @@
     </row>
     <row r="38" spans="1:21" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="17" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D38" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="E38" s="15" t="s">
         <v>45</v>
-      </c>
-      <c r="E38" s="15" t="s">
-        <v>46</v>
       </c>
       <c r="F38" s="13"/>
       <c r="G38" s="13"/>
       <c r="H38" s="17" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="I38" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="J38" s="25" t="s">
-        <v>137</v>
+        <v>106</v>
+      </c>
+      <c r="J38" s="15" t="s">
+        <v>130</v>
       </c>
       <c r="K38" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="L38" s="25" t="s">
-        <v>105</v>
+      <c r="L38" s="15" t="s">
+        <v>98</v>
       </c>
       <c r="M38" s="13"/>
       <c r="N38" s="13"/>
@@ -2892,36 +2881,36 @@
     </row>
     <row r="39" spans="1:21" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="17" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="D39" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="E39" s="15" t="s">
         <v>45</v>
-      </c>
-      <c r="E39" s="15" t="s">
-        <v>46</v>
       </c>
       <c r="F39" s="13"/>
       <c r="G39" s="13"/>
       <c r="H39" s="17" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="I39" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="J39" s="25" t="s">
-        <v>141</v>
+        <v>106</v>
+      </c>
+      <c r="J39" s="15" t="s">
+        <v>134</v>
       </c>
       <c r="K39" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="L39" s="25" t="s">
-        <v>105</v>
+      <c r="L39" s="15" t="s">
+        <v>98</v>
       </c>
       <c r="M39" s="13"/>
       <c r="N39" s="13"/>
@@ -2935,13 +2924,13 @@
     </row>
     <row r="40" spans="1:21" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="17" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="C40" s="15" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="D40" s="15" t="s">
         <v>19</v>
@@ -2952,19 +2941,19 @@
       <c r="F40" s="13"/>
       <c r="G40" s="13"/>
       <c r="H40" s="17" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="I40" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="J40" s="25" t="s">
-        <v>144</v>
+        <v>106</v>
+      </c>
+      <c r="J40" s="15" t="s">
+        <v>137</v>
       </c>
       <c r="K40" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="L40" s="25" t="s">
-        <v>98</v>
+        <v>44</v>
+      </c>
+      <c r="L40" s="15" t="s">
+        <v>91</v>
       </c>
       <c r="M40" s="13"/>
       <c r="N40" s="13"/>
@@ -2978,13 +2967,13 @@
     </row>
     <row r="41" spans="1:21" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="15" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="B41" s="15" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="C41" s="15" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="D41" s="15" t="s">
         <v>19</v>
@@ -2995,19 +2984,19 @@
       <c r="F41" s="13"/>
       <c r="G41" s="13"/>
       <c r="H41" s="17" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="I41" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="J41" s="25" t="s">
-        <v>147</v>
+        <v>106</v>
+      </c>
+      <c r="J41" s="15" t="s">
+        <v>140</v>
       </c>
       <c r="K41" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="L41" s="25" t="s">
-        <v>100</v>
+      <c r="L41" s="15" t="s">
+        <v>93</v>
       </c>
       <c r="M41" s="13"/>
       <c r="N41" s="13"/>
@@ -3021,63 +3010,63 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.3">
       <c r="H42" s="15" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="I42" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="J42" s="25" t="s">
-        <v>148</v>
+        <v>106</v>
+      </c>
+      <c r="J42" s="15" t="s">
+        <v>141</v>
       </c>
       <c r="K42" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="L42" s="25" t="s">
-        <v>100</v>
+      <c r="L42" s="15" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B43" s="22" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B44" s="21" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="C44" s="21" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="I44" s="22" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="J44" s="23" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B45" s="6" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="C45" s="20" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="I45" s="21" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="J45" s="21" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.3">
       <c r="I46" s="6" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="J46" s="20" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
     </row>
     <row r="48" spans="1:21" ht="36.6" x14ac:dyDescent="0.7">
@@ -3085,5 +3074,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>